<commit_message>
Update dashboard to show typical day patterns as percentages of maximum
Modify preprocessing script to calculate and save typical day averages as percentages of maximum values (0-100%), regenerate data file, and update app to use percentage data directly.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 8877ae72-82e6-4518-9133-e997a155a908
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 63866c15-3fdb-4f60-abad-e6a2544e6bcd
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/296373d1-a774-4ae0-bc03-ad5165af73dc/8877ae72-82e6-4518-9133-e997a155a908/vwfBUC0
</commit_message>
<xml_diff>
--- a/attached_assets/typical_day_averages.xlsx
+++ b/attached_assets/typical_day_averages.xlsx
@@ -472,19 +472,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1516.758333333333</v>
+        <v>78.01050935212331</v>
       </c>
       <c r="C2" t="n">
-        <v>5.683333333333334</v>
+        <v>18.28908554572272</v>
       </c>
       <c r="D2" t="n">
-        <v>66.79916666666666</v>
+        <v>97.59539289453818</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2</v>
+        <v>9.922041105598867</v>
       </c>
       <c r="F2" t="n">
-        <v>22.7475</v>
+        <v>99.16085440278989</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -495,19 +495,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1575.522123893805</v>
+        <v>81.03287167071981</v>
       </c>
       <c r="C3" t="n">
-        <v>4.946902654867257</v>
+        <v>15.91923621839825</v>
       </c>
       <c r="D3" t="n">
-        <v>66.80530973451327</v>
+        <v>97.60436808315183</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1902654867256637</v>
+        <v>9.439109901344054</v>
       </c>
       <c r="F3" t="n">
-        <v>22.78318584070797</v>
+        <v>99.31641604493447</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -518,19 +518,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1944.3</v>
+        <v>100</v>
       </c>
       <c r="C4" t="n">
-        <v>5.525</v>
+        <v>17.77956556717619</v>
       </c>
       <c r="D4" t="n">
-        <v>68.44500000000001</v>
+        <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>0.33</v>
+        <v>16.37136782423813</v>
       </c>
       <c r="F4" t="n">
-        <v>22.94</v>
+        <v>100</v>
       </c>
       <c r="G4" t="inlineStr"/>
     </row>
@@ -866,19 +866,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1213.036144578313</v>
+        <v>62.38935064436112</v>
       </c>
       <c r="C30" t="n">
-        <v>21.63253012048193</v>
+        <v>69.61393441828456</v>
       </c>
       <c r="D30" t="n">
-        <v>61.17650602409638</v>
+        <v>89.3805333100977</v>
       </c>
       <c r="E30" t="n">
-        <v>0.2198795180722891</v>
+        <v>10.90826808296261</v>
       </c>
       <c r="F30" t="n">
-        <v>22.26024096385542</v>
+        <v>97.03679583197658</v>
       </c>
       <c r="G30" t="inlineStr"/>
     </row>
@@ -889,19 +889,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1399.9</v>
+        <v>72.00020572956849</v>
       </c>
       <c r="C31" t="n">
-        <v>17.33</v>
+        <v>55.7683024939662</v>
       </c>
       <c r="D31" t="n">
-        <v>60.94199999999999</v>
+        <v>89.03791365329825</v>
       </c>
       <c r="E31" t="n">
-        <v>0.2656666666666667</v>
+        <v>13.1797779352705</v>
       </c>
       <c r="F31" t="n">
-        <v>22.04233333333333</v>
+        <v>96.08689334495787</v>
       </c>
       <c r="G31" t="inlineStr"/>
     </row>
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1360.533333333333</v>
+        <v>69.97548389308919</v>
       </c>
       <c r="C32" t="n">
-        <v>14.08</v>
+        <v>45.30973451327434</v>
       </c>
       <c r="D32" t="n">
-        <v>61.01733333333333</v>
+        <v>89.14797769498624</v>
       </c>
       <c r="E32" t="n">
-        <v>0.225</v>
+        <v>11.16229624379872</v>
       </c>
       <c r="F32" t="n">
-        <v>22.07733333333333</v>
+        <v>96.23946527172333</v>
       </c>
       <c r="G32" t="inlineStr"/>
     </row>
@@ -935,19 +935,19 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1310.456666666667</v>
+        <v>67.39992113699876</v>
       </c>
       <c r="C33" t="n">
-        <v>12.42333333333333</v>
+        <v>39.97854652721909</v>
       </c>
       <c r="D33" t="n">
-        <v>60.353</v>
+        <v>88.1773686901892</v>
       </c>
       <c r="E33" t="n">
-        <v>0.1913333333333333</v>
+        <v>9.492085991022915</v>
       </c>
       <c r="F33" t="n">
-        <v>22.18733333333333</v>
+        <v>96.71897704155768</v>
       </c>
       <c r="G33" t="inlineStr"/>
     </row>
@@ -958,19 +958,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1367.593333333333</v>
+        <v>70.33859658146034</v>
       </c>
       <c r="C34" t="n">
-        <v>19.25</v>
+        <v>61.94690265486725</v>
       </c>
       <c r="D34" t="n">
-        <v>60.54166666666666</v>
+        <v>88.45301580344314</v>
       </c>
       <c r="E34" t="n">
-        <v>0.379</v>
+        <v>18.80226789510985</v>
       </c>
       <c r="F34" t="n">
-        <v>22.242</v>
+        <v>96.95727986050566</v>
       </c>
       <c r="G34" t="inlineStr"/>
     </row>
@@ -981,19 +981,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1393.33</v>
+        <v>71.66229491333642</v>
       </c>
       <c r="C35" t="n">
-        <v>21.35</v>
+        <v>68.70474658085278</v>
       </c>
       <c r="D35" t="n">
-        <v>60.843</v>
+        <v>88.89327197019504</v>
       </c>
       <c r="E35" t="n">
-        <v>0.5589999999999999</v>
+        <v>27.73210489014883</v>
       </c>
       <c r="F35" t="n">
-        <v>22.20166666666667</v>
+        <v>96.78145887823308</v>
       </c>
       <c r="G35" t="inlineStr"/>
     </row>
@@ -1004,19 +1004,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1308.641025641026</v>
+        <v>67.30653837581781</v>
       </c>
       <c r="C36" t="n">
-        <v>17.20797720797721</v>
+        <v>55.37563059686954</v>
       </c>
       <c r="D36" t="n">
-        <v>61.44729344729345</v>
+        <v>89.77616107428365</v>
       </c>
       <c r="E36" t="n">
-        <v>0.4774928774928775</v>
+        <v>23.68851979057507</v>
       </c>
       <c r="F36" t="n">
-        <v>22.11595441595442</v>
+        <v>96.40782221427384</v>
       </c>
       <c r="G36" t="inlineStr"/>
     </row>
@@ -1027,19 +1027,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1236.280555555556</v>
+        <v>63.58486630435404</v>
       </c>
       <c r="C37" t="n">
-        <v>15.525</v>
+        <v>49.9597747385358</v>
       </c>
       <c r="D37" t="n">
-        <v>61.51944444444445</v>
+        <v>89.88157563656138</v>
       </c>
       <c r="E37" t="n">
-        <v>0.4188888888888889</v>
+        <v>20.78116387117096</v>
       </c>
       <c r="F37" t="n">
-        <v>22.08333333333333</v>
+        <v>96.26562045916886</v>
       </c>
       <c r="G37" t="inlineStr"/>
     </row>
@@ -1050,19 +1050,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1169.466666666667</v>
+        <v>60.14846817192134</v>
       </c>
       <c r="C38" t="n">
-        <v>13.64166666666667</v>
+        <v>43.89916867792974</v>
       </c>
       <c r="D38" t="n">
-        <v>61.41388888888889</v>
+        <v>89.72735610912248</v>
       </c>
       <c r="E38" t="n">
-        <v>0.37</v>
+        <v>18.3557760453579</v>
       </c>
       <c r="F38" t="n">
-        <v>22.02972222222222</v>
+        <v>96.03191901579</v>
       </c>
       <c r="G38" t="inlineStr"/>
     </row>
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1124.227777777778</v>
+        <v>57.82172389948968</v>
       </c>
       <c r="C39" t="n">
-        <v>12.46111111111111</v>
+        <v>40.10011620631089</v>
       </c>
       <c r="D39" t="n">
-        <v>61.29527777777778</v>
+        <v>89.55406206118455</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3458333333333333</v>
+        <v>17.15686274509804</v>
       </c>
       <c r="F39" t="n">
-        <v>22.0125</v>
+        <v>95.95684394071492</v>
       </c>
       <c r="G39" t="inlineStr"/>
     </row>
@@ -1096,19 +1096,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1069.386111111111</v>
+        <v>55.00108579494477</v>
       </c>
       <c r="C40" t="n">
-        <v>11.08888888888889</v>
+        <v>35.684276392241</v>
       </c>
       <c r="D40" t="n">
-        <v>61.11222222222223</v>
+        <v>89.28661293333658</v>
       </c>
       <c r="E40" t="n">
-        <v>0.3152777777777778</v>
+        <v>15.64099535396488</v>
       </c>
       <c r="F40" t="n">
-        <v>21.97166666666667</v>
+        <v>95.77884335948853</v>
       </c>
       <c r="G40" t="inlineStr"/>
     </row>
@@ -1119,19 +1119,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1068.97311827957</v>
+        <v>54.97984458568996</v>
       </c>
       <c r="C41" t="n">
-        <v>10.10483870967742</v>
+        <v>32.5175823320271</v>
       </c>
       <c r="D41" t="n">
-        <v>61.07177419354839</v>
+        <v>89.2275172672195</v>
       </c>
       <c r="E41" t="n">
-        <v>0.2889784946236559</v>
+        <v>14.33628251144998</v>
       </c>
       <c r="F41" t="n">
-        <v>21.97043010752688</v>
+        <v>95.77345295347376</v>
       </c>
       <c r="G41" t="inlineStr"/>
     </row>
@@ -1142,19 +1142,19 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1018.919047619048</v>
+        <v>52.40544399624789</v>
       </c>
       <c r="C42" t="n">
-        <v>8.316666666666666</v>
+        <v>26.76320729418075</v>
       </c>
       <c r="D42" t="n">
-        <v>60.79833333333333</v>
+        <v>88.82801275963668</v>
       </c>
       <c r="E42" t="n">
-        <v>0.2173809523809524</v>
+        <v>10.7843137254902</v>
       </c>
       <c r="F42" t="n">
-        <v>21.94952380952381</v>
+        <v>95.68231826296343</v>
       </c>
       <c r="G42" t="inlineStr"/>
     </row>
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1016.861904761905</v>
+        <v>52.29964021817131</v>
       </c>
       <c r="C43" t="n">
-        <v>7.930952380952381</v>
+        <v>25.52197065471402</v>
       </c>
       <c r="D43" t="n">
-        <v>60.64928571428572</v>
+        <v>88.61025014871167</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1980952380952381</v>
+        <v>9.827545476021735</v>
       </c>
       <c r="F43" t="n">
-        <v>21.9097619047619</v>
+        <v>95.50898825092375</v>
       </c>
       <c r="G43" t="inlineStr"/>
     </row>
@@ -1188,19 +1188,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1017.759523809524</v>
+        <v>52.34580691300334</v>
       </c>
       <c r="C44" t="n">
-        <v>7.638095238095238</v>
+        <v>24.57955024326706</v>
       </c>
       <c r="D44" t="n">
-        <v>60.54547619047619</v>
+        <v>88.45858162097477</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1866666666666667</v>
+        <v>9.260571698558943</v>
       </c>
       <c r="F44" t="n">
-        <v>21.91047619047619</v>
+        <v>95.51210196371487</v>
       </c>
       <c r="G44" t="inlineStr"/>
     </row>
@@ -1211,19 +1211,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>959.0383795309168</v>
+        <v>49.32563799469818</v>
       </c>
       <c r="C45" t="n">
-        <v>7.522388059701493</v>
+        <v>24.2072021229332</v>
       </c>
       <c r="D45" t="n">
-        <v>60.79957356076759</v>
+        <v>88.82982476553084</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1618336886993604</v>
+        <v>8.028602557728721</v>
       </c>
       <c r="F45" t="n">
-        <v>21.80319829424307</v>
+        <v>95.04445638292532</v>
       </c>
       <c r="G45" t="inlineStr"/>
     </row>
@@ -1234,19 +1234,19 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>950.9958333333333</v>
+        <v>48.91199060501637</v>
       </c>
       <c r="C46" t="n">
-        <v>8.345833333333333</v>
+        <v>26.85706623759721</v>
       </c>
       <c r="D46" t="n">
-        <v>60.68395833333333</v>
+        <v>88.6609077848394</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1658333333333334</v>
+        <v>8.227025750059063</v>
       </c>
       <c r="F46" t="n">
-        <v>21.815625</v>
+        <v>95.09862685265912</v>
       </c>
       <c r="G46" t="inlineStr"/>
     </row>
@@ -1257,19 +1257,19 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>936.0458333333333</v>
+        <v>48.14307634281404</v>
       </c>
       <c r="C47" t="n">
-        <v>8.345833333333333</v>
+        <v>26.85706623759721</v>
       </c>
       <c r="D47" t="n">
-        <v>60.6525</v>
+        <v>88.614946307254</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1475</v>
+        <v>7.317505315379163</v>
       </c>
       <c r="F47" t="n">
-        <v>21.85125</v>
+        <v>95.25392327811684</v>
       </c>
       <c r="G47" t="inlineStr"/>
     </row>
@@ -1280,19 +1280,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>928.69375</v>
+        <v>47.76494110991102</v>
       </c>
       <c r="C48" t="n">
-        <v>12.60625</v>
+        <v>40.56717618664521</v>
       </c>
       <c r="D48" t="n">
-        <v>60.80833333333333</v>
+        <v>88.84262303065721</v>
       </c>
       <c r="E48" t="n">
-        <v>0.491875</v>
+        <v>24.40201984408221</v>
       </c>
       <c r="F48" t="n">
-        <v>21.865625</v>
+        <v>95.31658674803838</v>
       </c>
       <c r="G48" t="inlineStr"/>
     </row>
@@ -1303,19 +1303,19 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>959.7349137931035</v>
+        <v>49.36146241799638</v>
       </c>
       <c r="C49" t="n">
-        <v>16.28879310344828</v>
+        <v>52.41767692179656</v>
       </c>
       <c r="D49" t="n">
-        <v>61.33211206896551</v>
+        <v>89.60787795889475</v>
       </c>
       <c r="E49" t="n">
-        <v>1.019612068965517</v>
+        <v>50.58316430020285</v>
       </c>
       <c r="F49" t="n">
-        <v>21.88254310344828</v>
+        <v>95.39033610919041</v>
       </c>
       <c r="G49" t="inlineStr"/>
     </row>
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>985.347619047619</v>
+        <v>50.67878511791488</v>
       </c>
       <c r="C50" t="n">
-        <v>20.94761904761905</v>
+        <v>67.40987625943377</v>
       </c>
       <c r="D50" t="n">
-        <v>62.30595238095238</v>
+        <v>91.03068504777906</v>
       </c>
       <c r="E50" t="n">
-        <v>1.043809523809524</v>
+        <v>51.78360500826836</v>
       </c>
       <c r="F50" t="n">
-        <v>21.90595238095238</v>
+        <v>95.49238178270437</v>
       </c>
       <c r="G50" t="inlineStr"/>
     </row>
@@ -1349,19 +1349,19 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>984.2214285714285</v>
+        <v>50.62086244774101</v>
       </c>
       <c r="C51" t="n">
-        <v>24.27857142857143</v>
+        <v>78.12895069532237</v>
       </c>
       <c r="D51" t="n">
-        <v>62.10952380952381</v>
+        <v>90.7436975813044</v>
       </c>
       <c r="E51" t="n">
-        <v>1.06952380952381</v>
+        <v>53.05929600755965</v>
       </c>
       <c r="F51" t="n">
-        <v>21.97619047619047</v>
+        <v>95.79856354049903</v>
       </c>
       <c r="G51" t="inlineStr"/>
     </row>
@@ -1372,19 +1372,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>972.1261904761905</v>
+        <v>49.99877541923522</v>
       </c>
       <c r="C52" t="n">
-        <v>21.34047619047619</v>
+        <v>68.67409876259435</v>
       </c>
       <c r="D52" t="n">
-        <v>62.03309523809524</v>
+        <v>90.6320333670761</v>
       </c>
       <c r="E52" t="n">
-        <v>0.9352380952380953</v>
+        <v>46.39735412237185</v>
       </c>
       <c r="F52" t="n">
-        <v>22.00714285714286</v>
+        <v>95.93349109478142</v>
       </c>
       <c r="G52" t="inlineStr"/>
     </row>
@@ -1395,19 +1395,19 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>941.2690476190476</v>
+        <v>48.41171874808659</v>
       </c>
       <c r="C53" t="n">
-        <v>19.28809523809524</v>
+        <v>62.06949392790101</v>
       </c>
       <c r="D53" t="n">
-        <v>61.97428571428571</v>
+        <v>90.54611105893156</v>
       </c>
       <c r="E53" t="n">
-        <v>0.8383333333333334</v>
+        <v>41.58988896763525</v>
       </c>
       <c r="F53" t="n">
-        <v>22.00785714285714</v>
+        <v>95.93660480757256</v>
       </c>
       <c r="G53" t="inlineStr"/>
     </row>
@@ -1418,19 +1418,19 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>920.2333333333333</v>
+        <v>47.32980164240772</v>
       </c>
       <c r="C54" t="n">
-        <v>17.24761904761905</v>
+        <v>55.50319886603072</v>
       </c>
       <c r="D54" t="n">
-        <v>61.90809523809524</v>
+        <v>90.4494049793195</v>
       </c>
       <c r="E54" t="n">
-        <v>0.7509523809523809</v>
+        <v>37.25490196078432</v>
       </c>
       <c r="F54" t="n">
-        <v>22.01190476190476</v>
+        <v>95.95424918005564</v>
       </c>
       <c r="G54" t="inlineStr"/>
     </row>
@@ -1441,19 +1441,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>918.4285714285714</v>
+        <v>47.23697842043777</v>
       </c>
       <c r="C55" t="n">
-        <v>19.90952380952381</v>
+        <v>64.06926406926407</v>
       </c>
       <c r="D55" t="n">
-        <v>62.03428571428572</v>
+        <v>90.63377268505472</v>
       </c>
       <c r="E55" t="n">
-        <v>0.7380952380952381</v>
+        <v>36.61705646113867</v>
       </c>
       <c r="F55" t="n">
-        <v>22.07833333333333</v>
+        <v>96.24382446963094</v>
       </c>
       <c r="G55" t="inlineStr"/>
     </row>
@@ -1464,19 +1464,19 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>897.0358851674641</v>
+        <v>46.13670139214443</v>
       </c>
       <c r="C56" t="n">
-        <v>18.72142857142857</v>
+        <v>60.24594874152397</v>
       </c>
       <c r="D56" t="n">
-        <v>62.38928571428571</v>
+        <v>91.15243730628345</v>
       </c>
       <c r="E56" t="n">
-        <v>0.638095238095238</v>
+        <v>31.65603590833924</v>
       </c>
       <c r="F56" t="n">
-        <v>22.11404761904762</v>
+        <v>96.39951010918753</v>
       </c>
       <c r="G56" t="inlineStr"/>
     </row>
@@ -1487,19 +1487,19 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>906.1214285714286</v>
+        <v>46.60399262312548</v>
       </c>
       <c r="C57" t="n">
-        <v>17.15476190476191</v>
+        <v>55.20438263801096</v>
       </c>
       <c r="D57" t="n">
-        <v>62.54071428571428</v>
+        <v>91.37367855316572</v>
       </c>
       <c r="E57" t="n">
-        <v>1.25</v>
+        <v>62.01275690999292</v>
       </c>
       <c r="F57" t="n">
-        <v>22.13047619047619</v>
+        <v>96.47112550338356</v>
       </c>
       <c r="G57" t="inlineStr"/>
     </row>
@@ -1510,19 +1510,19 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>918.2357142857143</v>
+        <v>47.22705931624309</v>
       </c>
       <c r="C58" t="n">
-        <v>19.04761904761905</v>
+        <v>61.29563651687545</v>
       </c>
       <c r="D58" t="n">
-        <v>62.3652380952381</v>
+        <v>91.11730308311505</v>
       </c>
       <c r="E58" t="n">
-        <v>2.015714285714286</v>
+        <v>100</v>
       </c>
       <c r="F58" t="n">
-        <v>22.11476190476191</v>
+        <v>96.40262382197868</v>
       </c>
       <c r="G58" t="inlineStr"/>
     </row>
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>936.7119047619047</v>
+        <v>48.17733398970863</v>
       </c>
       <c r="C59" t="n">
-        <v>17.1047619047619</v>
+        <v>55.04348159215415</v>
       </c>
       <c r="D59" t="n">
-        <v>62.69166666666667</v>
+        <v>91.59422407285655</v>
       </c>
       <c r="E59" t="n">
-        <v>1.729761904761905</v>
+        <v>85.81384360973307</v>
       </c>
       <c r="F59" t="n">
-        <v>22.18452380952381</v>
+        <v>96.70672977124592</v>
       </c>
       <c r="G59" t="inlineStr"/>
     </row>
@@ -1556,19 +1556,19 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>927.7857142857143</v>
+        <v>47.71823866099441</v>
       </c>
       <c r="C60" t="n">
-        <v>14.55714285714286</v>
+        <v>46.84519020802207</v>
       </c>
       <c r="D60" t="n">
-        <v>62.9247619047619</v>
+        <v>91.93478253307312</v>
       </c>
       <c r="E60" t="n">
-        <v>1.391190476190476</v>
+        <v>69.01724545239783</v>
       </c>
       <c r="F60" t="n">
-        <v>22.18166666666666</v>
+        <v>96.69427492008137</v>
       </c>
       <c r="G60" t="inlineStr"/>
     </row>
@@ -1579,19 +1579,19 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>936.7952380952381</v>
+        <v>48.18162002238534</v>
       </c>
       <c r="C61" t="n">
-        <v>13.33333333333333</v>
+        <v>42.90694556181282</v>
       </c>
       <c r="D61" t="n">
-        <v>62.805</v>
+        <v>91.75980714442252</v>
       </c>
       <c r="E61" t="n">
-        <v>1.240952380952381</v>
+        <v>61.56390266950154</v>
       </c>
       <c r="F61" t="n">
-        <v>22.18166666666666</v>
+        <v>96.69427492008137</v>
       </c>
       <c r="G61" t="inlineStr"/>
     </row>
@@ -1602,19 +1602,19 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>955.9761904761905</v>
+        <v>49.16814228648822</v>
       </c>
       <c r="C62" t="n">
-        <v>12.47380952380952</v>
+        <v>40.14097996398881</v>
       </c>
       <c r="D62" t="n">
-        <v>62.69309523809523</v>
+        <v>91.5963112544309</v>
       </c>
       <c r="E62" t="n">
-        <v>1.064285714285714</v>
+        <v>52.79943302622254</v>
       </c>
       <c r="F62" t="n">
-        <v>22.18357142857143</v>
+        <v>96.70257815419107</v>
       </c>
       <c r="G62" t="inlineStr"/>
     </row>
@@ -1625,19 +1625,19 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>952.1674641148326</v>
+        <v>48.97225037879096</v>
       </c>
       <c r="C63" t="n">
-        <v>11.21428571428571</v>
+        <v>36.08780599931043</v>
       </c>
       <c r="D63" t="n">
-        <v>62.72785714285715</v>
+        <v>91.64709933940702</v>
       </c>
       <c r="E63" t="n">
-        <v>0.9097619047619048</v>
+        <v>45.1334750767777</v>
       </c>
       <c r="F63" t="n">
-        <v>22.14785714285714</v>
+        <v>96.54689251463446</v>
       </c>
       <c r="G63" t="inlineStr"/>
     </row>
@@ -1648,19 +1648,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>943.8190476190476</v>
+        <v>48.54287134799402</v>
       </c>
       <c r="C64" t="n">
-        <v>10.81666666666667</v>
+        <v>34.80825958702065</v>
       </c>
       <c r="D64" t="n">
-        <v>62.74547619047619</v>
+        <v>91.67284124549082</v>
       </c>
       <c r="E64" t="n">
-        <v>0.8099999999999999</v>
+        <v>40.18426647767541</v>
       </c>
       <c r="F64" t="n">
-        <v>22.17714285714286</v>
+        <v>96.67455473907089</v>
       </c>
       <c r="G64" t="inlineStr"/>
     </row>
@@ -1671,19 +1671,19 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>972.491646778043</v>
+        <v>50.01757171105503</v>
       </c>
       <c r="C65" t="n">
-        <v>10.1452380952381</v>
+        <v>32.64758839980079</v>
       </c>
       <c r="D65" t="n">
-        <v>62.93119047619047</v>
+        <v>91.94417485015775</v>
       </c>
       <c r="E65" t="n">
-        <v>0.7366666666666666</v>
+        <v>36.54618473895582</v>
       </c>
       <c r="F65" t="n">
-        <v>22.16738095238095</v>
+        <v>96.63200066425874</v>
       </c>
       <c r="G65" t="inlineStr"/>
     </row>
@@ -1694,19 +1694,19 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1035.009523809524</v>
+        <v>53.23301567708295</v>
       </c>
       <c r="C66" t="n">
-        <v>10.81904761904762</v>
+        <v>34.81592154158526</v>
       </c>
       <c r="D66" t="n">
-        <v>63.21714285714286</v>
+        <v>92.36195902862569</v>
       </c>
       <c r="E66" t="n">
-        <v>0.7107142857142857</v>
+        <v>35.2586817859674</v>
       </c>
       <c r="F66" t="n">
-        <v>22.17619047619048</v>
+        <v>96.67040312201604</v>
       </c>
       <c r="G66" t="inlineStr"/>
     </row>
@@ -1717,19 +1717,19 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1023.895261845387</v>
+        <v>52.66138259761285</v>
       </c>
       <c r="C67" t="n">
-        <v>11</v>
+        <v>35.39823008849557</v>
       </c>
       <c r="D67" t="n">
-        <v>62.8219451371571</v>
+        <v>91.78456444905704</v>
       </c>
       <c r="E67" t="n">
-        <v>0.6718204488778055</v>
+        <v>33.32915054673734</v>
       </c>
       <c r="F67" t="n">
-        <v>22.2002493765586</v>
+        <v>96.77528063015957</v>
       </c>
       <c r="G67" t="inlineStr"/>
     </row>
@@ -1740,19 +1740,19 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>952.275</v>
+        <v>48.97778120660392</v>
       </c>
       <c r="C68" t="n">
-        <v>7.411111111111111</v>
+        <v>23.84911057477429</v>
       </c>
       <c r="D68" t="n">
-        <v>61.83972222222222</v>
+        <v>90.34951015007994</v>
       </c>
       <c r="E68" t="n">
-        <v>0.5225</v>
+        <v>25.92133238837704</v>
       </c>
       <c r="F68" t="n">
-        <v>22.19277777777778</v>
+        <v>96.74271045238788</v>
       </c>
       <c r="G68" t="inlineStr"/>
     </row>
@@ -1763,19 +1763,19 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>981.3083333333333</v>
+        <v>50.47103499117077</v>
       </c>
       <c r="C69" t="n">
-        <v>7.2</v>
+        <v>23.16975060337892</v>
       </c>
       <c r="D69" t="n">
-        <v>61.87805555555555</v>
+        <v>90.40551618899195</v>
       </c>
       <c r="E69" t="n">
-        <v>0.5241666666666667</v>
+        <v>26.00401606425703</v>
       </c>
       <c r="F69" t="n">
-        <v>22.18694444444445</v>
+        <v>96.71728179792697</v>
       </c>
       <c r="G69" t="inlineStr"/>
     </row>
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>990.35</v>
+        <v>50.93606953659415</v>
       </c>
       <c r="C70" t="n">
-        <v>7.552777777777778</v>
+        <v>24.30499687136855</v>
       </c>
       <c r="D70" t="n">
-        <v>61.86333333333333</v>
+        <v>90.38400662332285</v>
       </c>
       <c r="E70" t="n">
-        <v>0.53</v>
+        <v>26.293408929837</v>
       </c>
       <c r="F70" t="n">
-        <v>22.1825</v>
+        <v>96.69790758500437</v>
       </c>
       <c r="G70" t="inlineStr"/>
     </row>
@@ -1809,19 +1809,19 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>982.2638888888889</v>
+        <v>50.52018149919708</v>
       </c>
       <c r="C71" t="n">
-        <v>8.316666666666666</v>
+        <v>26.76320729418075</v>
       </c>
       <c r="D71" t="n">
-        <v>61.82694444444444</v>
+        <v>90.33084147044261</v>
       </c>
       <c r="E71" t="n">
-        <v>0.4844444444444445</v>
+        <v>24.03338845578392</v>
       </c>
       <c r="F71" t="n">
-        <v>22.22333333333333</v>
+        <v>96.87590816623074</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
@@ -1832,19 +1832,19 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1015.55</v>
+        <v>52.23216581803219</v>
       </c>
       <c r="C72" t="n">
-        <v>8.791666666666666</v>
+        <v>28.29176722982033</v>
       </c>
       <c r="D72" t="n">
-        <v>62.27916666666667</v>
+        <v>90.99155039325979</v>
       </c>
       <c r="E72" t="n">
-        <v>0.4175</v>
+        <v>20.71226080793764</v>
       </c>
       <c r="F72" t="n">
-        <v>22.21277777777778</v>
+        <v>96.82989441053958</v>
       </c>
       <c r="G72" t="inlineStr"/>
     </row>
@@ -1855,19 +1855,19 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1029.147222222222</v>
+        <v>52.93150348311588</v>
       </c>
       <c r="C73" t="n">
-        <v>11.40277777777778</v>
+        <v>36.69437740234201</v>
       </c>
       <c r="D73" t="n">
-        <v>62.43638888888889</v>
+        <v>91.22125632097141</v>
       </c>
       <c r="E73" t="n">
-        <v>0.3941666666666667</v>
+        <v>19.55468934561777</v>
       </c>
       <c r="F73" t="n">
-        <v>22.22583333333333</v>
+        <v>96.88680616099971</v>
       </c>
       <c r="G73" t="inlineStr"/>
     </row>
@@ -1878,19 +1878,19 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1066.641666666667</v>
+        <v>54.85993245212502</v>
       </c>
       <c r="C74" t="n">
-        <v>23.35</v>
+        <v>75.1407884151247</v>
       </c>
       <c r="D74" t="n">
-        <v>63.07083333333333</v>
+        <v>92.14819684905154</v>
       </c>
       <c r="E74" t="n">
-        <v>0.3486111111111111</v>
+        <v>17.29466887156469</v>
       </c>
       <c r="F74" t="n">
-        <v>22.27194444444444</v>
+        <v>97.0878136200717</v>
       </c>
       <c r="G74" t="inlineStr"/>
     </row>
@@ -1901,19 +1901,19 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1101.669444444444</v>
+        <v>56.66149485390343</v>
       </c>
       <c r="C75" t="n">
-        <v>21.63333333333333</v>
+        <v>69.6165191740413</v>
       </c>
       <c r="D75" t="n">
-        <v>63.51833333333333</v>
+        <v>92.80200647722013</v>
       </c>
       <c r="E75" t="n">
-        <v>0.3041666666666666</v>
+        <v>15.08977084809827</v>
       </c>
       <c r="F75" t="n">
-        <v>22.355</v>
+        <v>97.44986922406278</v>
       </c>
       <c r="G75" t="inlineStr"/>
     </row>
@@ -1924,19 +1924,19 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1170.630555555555</v>
+        <v>60.20832976163943</v>
       </c>
       <c r="C76" t="n">
-        <v>20.09722222222222</v>
+        <v>64.67328148744078</v>
       </c>
       <c r="D76" t="n">
-        <v>63.61833333333333</v>
+        <v>92.94810918742542</v>
       </c>
       <c r="E76" t="n">
-        <v>0.2722222222222222</v>
+        <v>13.50500039373179</v>
       </c>
       <c r="F76" t="n">
-        <v>22.40611111111111</v>
+        <v>97.67267267267268</v>
       </c>
       <c r="G76" t="inlineStr"/>
     </row>
@@ -1947,19 +1947,19 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1240.986111111111</v>
+        <v>63.82688428283244</v>
       </c>
       <c r="C77" t="n">
-        <v>23.60555555555555</v>
+        <v>75.96317153839277</v>
       </c>
       <c r="D77" t="n">
-        <v>63.50472222222223</v>
+        <v>92.78212027499777</v>
       </c>
       <c r="E77" t="n">
-        <v>0.2911111111111111</v>
+        <v>14.44208205370502</v>
       </c>
       <c r="F77" t="n">
-        <v>22.48138888888889</v>
+        <v>98.00082340404923</v>
       </c>
       <c r="G77" t="inlineStr"/>
     </row>
@@ -1970,19 +1970,19 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1302.125</v>
+        <v>66.97140358998097</v>
       </c>
       <c r="C78" t="n">
-        <v>31.075</v>
+        <v>100</v>
       </c>
       <c r="D78" t="n">
-        <v>63.34805555555555</v>
+        <v>92.55322602900949</v>
       </c>
       <c r="E78" t="n">
-        <v>0.3997222222222223</v>
+        <v>19.83030159855107</v>
       </c>
       <c r="F78" t="n">
-        <v>22.53722222222222</v>
+        <v>98.24421195388938</v>
       </c>
       <c r="G78" t="inlineStr"/>
     </row>
@@ -1993,19 +1993,19 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1320.505555555555</v>
+        <v>67.91675953070799</v>
       </c>
       <c r="C79" t="n">
-        <v>23.90555555555556</v>
+        <v>76.92857781353356</v>
       </c>
       <c r="D79" t="n">
-        <v>63.43888888888889</v>
+        <v>92.68593599077929</v>
       </c>
       <c r="E79" t="n">
-        <v>0.3488888888888889</v>
+        <v>17.30844948421136</v>
       </c>
       <c r="F79" t="n">
-        <v>22.55916666666667</v>
+        <v>98.33987213019472</v>
       </c>
       <c r="G79" t="inlineStr"/>
     </row>
@@ -2016,19 +2016,19 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1361.897222222222</v>
+        <v>70.04563196123141</v>
       </c>
       <c r="C80" t="n">
-        <v>20.00555555555556</v>
+        <v>64.37829623670332</v>
       </c>
       <c r="D80" t="n">
-        <v>63.55277777777778</v>
+        <v>92.85233074406862</v>
       </c>
       <c r="E80" t="n">
-        <v>0.3255555555555555</v>
+        <v>16.15087802189149</v>
       </c>
       <c r="F80" t="n">
-        <v>22.53944444444445</v>
+        <v>98.25389906035069</v>
       </c>
       <c r="G80" t="inlineStr"/>
     </row>
@@ -2039,19 +2039,19 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1384.863888888889</v>
+        <v>71.22686256693355</v>
       </c>
       <c r="C81" t="n">
-        <v>17.08611111111111</v>
+        <v>54.98346294806472</v>
       </c>
       <c r="D81" t="n">
-        <v>63.47527777777778</v>
+        <v>92.73910114365954</v>
       </c>
       <c r="E81" t="n">
-        <v>0.2980555555555556</v>
+        <v>14.78659736987165</v>
       </c>
       <c r="F81" t="n">
-        <v>22.605</v>
+        <v>98.53966870095904</v>
       </c>
       <c r="G81" t="inlineStr"/>
     </row>
@@ -2062,19 +2062,19 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1426.255555555555</v>
+        <v>73.35573499745695</v>
       </c>
       <c r="C82" t="n">
-        <v>17.26666666666667</v>
+        <v>55.5644945025476</v>
       </c>
       <c r="D82" t="n">
-        <v>63.40916666666666</v>
+        <v>92.64251101857937</v>
       </c>
       <c r="E82" t="n">
-        <v>0.2916666666666667</v>
+        <v>14.46964327899835</v>
       </c>
       <c r="F82" t="n">
-        <v>22.62944444444445</v>
+        <v>98.64622687203334</v>
       </c>
       <c r="G82" t="inlineStr"/>
     </row>
@@ -2085,19 +2085,19 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1486.330555555556</v>
+        <v>76.44553595409946</v>
       </c>
       <c r="C83" t="n">
-        <v>19.07777777777778</v>
+        <v>61.39268794136051</v>
       </c>
       <c r="D83" t="n">
-        <v>63.17388888888888</v>
+        <v>92.2987638087353</v>
       </c>
       <c r="E83" t="n">
-        <v>0.3391666666666667</v>
+        <v>16.82612804157808</v>
       </c>
       <c r="F83" t="n">
-        <v>22.72833333333333</v>
+        <v>99.07730310956117</v>
       </c>
       <c r="G83" t="inlineStr"/>
     </row>
@@ -2108,19 +2108,19 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1519.947222222222</v>
+        <v>78.17452153588553</v>
       </c>
       <c r="C84" t="n">
-        <v>15.66388888888889</v>
+        <v>50.40672208813803</v>
       </c>
       <c r="D84" t="n">
-        <v>62.81055555555555</v>
+        <v>91.76792396165614</v>
       </c>
       <c r="E84" t="n">
-        <v>0.3075</v>
+        <v>15.25513819985826</v>
       </c>
       <c r="F84" t="n">
-        <v>22.76444444444445</v>
+        <v>99.23471858955732</v>
       </c>
       <c r="G84" t="inlineStr"/>
     </row>
@@ -2131,19 +2131,19 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>1446.920844327177</v>
+        <v>74.41860023284353</v>
       </c>
       <c r="C85" t="n">
-        <v>15.30870712401055</v>
+        <v>49.26373973937427</v>
       </c>
       <c r="D85" t="n">
-        <v>62.80395778364116</v>
+        <v>91.75828443807606</v>
       </c>
       <c r="E85" t="n">
-        <v>0.3113456464379947</v>
+        <v>15.44592151003518</v>
       </c>
       <c r="F85" t="n">
-        <v>22.79683377308707</v>
+        <v>99.37591008320433</v>
       </c>
       <c r="G85" t="inlineStr"/>
     </row>
@@ -2154,19 +2154,19 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>1390.088095238095</v>
+        <v>71.49555599640463</v>
       </c>
       <c r="C86" t="n">
-        <v>14.61904761904762</v>
+        <v>47.04440102670191</v>
       </c>
       <c r="D86" t="n">
-        <v>63.58976190476191</v>
+        <v>92.90636555593819</v>
       </c>
       <c r="E86" t="n">
-        <v>0.3323809523809524</v>
+        <v>16.48948736120954</v>
       </c>
       <c r="F86" t="n">
-        <v>22.75404761904762</v>
+        <v>99.18939677004195</v>
       </c>
       <c r="G86" t="inlineStr"/>
     </row>
@@ -2177,19 +2177,19 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1408.871428571429</v>
+        <v>72.46162776173577</v>
       </c>
       <c r="C87" t="n">
-        <v>13.45714285714286</v>
+        <v>43.30536719917252</v>
       </c>
       <c r="D87" t="n">
-        <v>64.0552380952381</v>
+        <v>93.58643888558417</v>
       </c>
       <c r="E87" t="n">
-        <v>0.3183333333333333</v>
+        <v>15.7925820930782</v>
       </c>
       <c r="F87" t="n">
-        <v>22.76047619047619</v>
+        <v>99.21742018516213</v>
       </c>
       <c r="G87" t="inlineStr"/>
     </row>
@@ -2200,19 +2200,19 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>1426.580952380952</v>
+        <v>73.37247093457555</v>
       </c>
       <c r="C88" t="n">
-        <v>11.56666666666667</v>
+        <v>37.22177527487262</v>
       </c>
       <c r="D88" t="n">
-        <v>63.9097619047619</v>
+        <v>93.37389422859506</v>
       </c>
       <c r="E88" t="n">
-        <v>0.3026190476190476</v>
+        <v>15.01299314906685</v>
       </c>
       <c r="F88" t="n">
-        <v>22.82666666666667</v>
+        <v>99.50595757047371</v>
       </c>
       <c r="G88" t="inlineStr"/>
     </row>
@@ -2223,19 +2223,19 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>1418.159523809524</v>
+        <v>72.93933671807457</v>
       </c>
       <c r="C89" t="n">
-        <v>11.00238095238095</v>
+        <v>35.40589204306019</v>
       </c>
       <c r="D89" t="n">
-        <v>63.91857142857143</v>
+        <v>93.38676518163696</v>
       </c>
       <c r="E89" t="n">
-        <v>1.193571428571429</v>
+        <v>59.21332388377037</v>
       </c>
       <c r="F89" t="n">
-        <v>22.7997619047619</v>
+        <v>99.3886743886744</v>
       </c>
       <c r="G89" t="inlineStr"/>
     </row>
@@ -2246,19 +2246,19 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1428.147619047619</v>
+        <v>73.45304834889775</v>
       </c>
       <c r="C90" t="n">
-        <v>10.21904761904762</v>
+        <v>32.88510899130368</v>
       </c>
       <c r="D90" t="n">
-        <v>63.93261904761905</v>
+        <v>93.40728913378486</v>
       </c>
       <c r="E90" t="n">
-        <v>1.312619047619048</v>
+        <v>65.11930073234113</v>
       </c>
       <c r="F90" t="n">
-        <v>22.85190476190476</v>
+        <v>99.61597542242703</v>
       </c>
       <c r="G90" t="inlineStr"/>
     </row>
@@ -2269,19 +2269,19 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1417.540476190476</v>
+        <v>72.90749761819042</v>
       </c>
       <c r="C91" t="n">
-        <v>9.616666666666667</v>
+        <v>30.9466344864575</v>
       </c>
       <c r="D91" t="n">
-        <v>63.58761904761904</v>
+        <v>92.90323478357665</v>
       </c>
       <c r="E91" t="n">
-        <v>0.9364285714285715</v>
+        <v>46.45641389085755</v>
       </c>
       <c r="F91" t="n">
-        <v>22.90642857142857</v>
+        <v>99.85365549881681</v>
       </c>
       <c r="G91" t="inlineStr"/>
     </row>
@@ -2292,19 +2292,19 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>1413.209523809524</v>
+        <v>72.6847463770778</v>
       </c>
       <c r="C92" t="n">
-        <v>21.73333333333333</v>
+        <v>69.93832126575489</v>
       </c>
       <c r="D92" t="n">
-        <v>63.51357142857143</v>
+        <v>92.79504920530562</v>
       </c>
       <c r="E92" t="n">
-        <v>0.8692857142857143</v>
+        <v>43.12544294826365</v>
       </c>
       <c r="F92" t="n">
-        <v>22.85333333333333</v>
+        <v>99.62220284800929</v>
       </c>
       <c r="G92" t="inlineStr"/>
     </row>
@@ -2315,19 +2315,19 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1433.401459854015</v>
+        <v>73.72326594939128</v>
       </c>
       <c r="C93" t="n">
-        <v>17.57664233576642</v>
+        <v>56.56200268951383</v>
       </c>
       <c r="D93" t="n">
-        <v>63.61313868613139</v>
+        <v>92.94051966707777</v>
       </c>
       <c r="E93" t="n">
-        <v>0.8124087591240875</v>
+        <v>40.30376551288882</v>
       </c>
       <c r="F93" t="n">
-        <v>22.81192214111922</v>
+        <v>99.44168326555895</v>
       </c>
       <c r="G93" t="inlineStr"/>
     </row>
@@ -2338,19 +2338,19 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1420.705705705706</v>
+        <v>73.07029294376926</v>
       </c>
       <c r="C94" t="n">
-        <v>16.59159159159159</v>
+        <v>53.39208879031888</v>
       </c>
       <c r="D94" t="n">
-        <v>64.87747747747748</v>
+        <v>94.78775290741103</v>
       </c>
       <c r="E94" t="n">
-        <v>0.8264264264264264</v>
+        <v>40.9991848687809</v>
       </c>
       <c r="F94" t="n">
-        <v>22.87477477477477</v>
+        <v>99.71567033467645</v>
       </c>
       <c r="G94" t="inlineStr"/>
     </row>
@@ -2361,19 +2361,19 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1433.162361623616</v>
+        <v>73.71096855545011</v>
       </c>
       <c r="C95" t="n">
-        <v>16.99630996309963</v>
+        <v>54.69448097538096</v>
       </c>
       <c r="D95" t="n">
-        <v>65.11070110701107</v>
+        <v>95.12849895099869</v>
       </c>
       <c r="E95" t="n">
-        <v>0.6461254612546126</v>
+        <v>32.05441692971147</v>
       </c>
       <c r="F95" t="n">
-        <v>22.80738007380074</v>
+        <v>99.42188349520812</v>
       </c>
       <c r="G95" t="inlineStr"/>
     </row>
@@ -2384,19 +2384,19 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>1449.454545454545</v>
+        <v>74.54891454274266</v>
       </c>
       <c r="C96" t="n">
-        <v>10.81818181818182</v>
+        <v>34.81313537628904</v>
       </c>
       <c r="D96" t="n">
-        <v>66.67878787878789</v>
+        <v>97.41951622293503</v>
       </c>
       <c r="E96" t="n">
-        <v>0.2568181818181818</v>
+        <v>12.74080278332582</v>
       </c>
       <c r="F96" t="n">
-        <v>22.78106060606061</v>
+        <v>99.30715172650658</v>
       </c>
       <c r="G96" t="inlineStr"/>
     </row>
@@ -2407,19 +2407,19 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1456.491666666667</v>
+        <v>74.91085052032437</v>
       </c>
       <c r="C97" t="n">
-        <v>6.266666666666667</v>
+        <v>20.16626441405202</v>
       </c>
       <c r="D97" t="n">
-        <v>66.76666666666667</v>
+        <v>97.54790951372146</v>
       </c>
       <c r="E97" t="n">
-        <v>0.2066666666666667</v>
+        <v>10.25277580911883</v>
       </c>
       <c r="F97" t="n">
-        <v>22.73833333333333</v>
+        <v>99.12089508863703</v>
       </c>
       <c r="G97" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update typical day heatmap to show percentage of range with new color scheme
Adjusted preprocessing script to normalize values between min and max, and updated app.py to use a pale grey to brown color scale for the typical day heatmap, changing the colorbar title to "% of Range".

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 8877ae72-82e6-4518-9133-e997a155a908
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4d3ed2a7-d3e6-4949-902a-f3654611450b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/296373d1-a774-4ae0-bc03-ad5165af73dc/8877ae72-82e6-4518-9133-e997a155a908/vwfBUC0
</commit_message>
<xml_diff>
--- a/attached_assets/typical_day_averages.xlsx
+++ b/attached_assets/typical_day_averages.xlsx
@@ -472,19 +472,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>78.01050935212331</v>
+        <v>59.1753731831981</v>
       </c>
       <c r="C2" t="n">
-        <v>18.28908554572272</v>
+        <v>2.818539248144917</v>
       </c>
       <c r="D2" t="n">
-        <v>97.59539289453818</v>
+        <v>79.66098203987467</v>
       </c>
       <c r="E2" t="n">
-        <v>9.922041105598867</v>
+        <v>2.810170139552668</v>
       </c>
       <c r="F2" t="n">
-        <v>99.16085440278989</v>
+        <v>83.06652787155836</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -495,19 +495,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81.03287167071981</v>
+        <v>64.78654516247178</v>
       </c>
       <c r="C3" t="n">
-        <v>15.91923621839825</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>97.60436808315183</v>
+        <v>79.73689736175564</v>
       </c>
       <c r="E3" t="n">
-        <v>9.439109901344054</v>
+        <v>2.289110358093259</v>
       </c>
       <c r="F3" t="n">
-        <v>99.31641604493447</v>
+        <v>86.20567171056281</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -521,13 +521,13 @@
         <v>100</v>
       </c>
       <c r="C4" t="n">
-        <v>17.77956556717619</v>
+        <v>2.212550487303025</v>
       </c>
       <c r="D4" t="n">
         <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>16.37136782423813</v>
+        <v>9.768686675587841</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -866,19 +866,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>62.38935064436112</v>
+        <v>30.17388402173788</v>
       </c>
       <c r="C30" t="n">
-        <v>69.61393441828456</v>
+        <v>63.86085923215126</v>
       </c>
       <c r="D30" t="n">
-        <v>89.3805333100977</v>
+        <v>10.17679219100817</v>
       </c>
       <c r="E30" t="n">
-        <v>10.90826808296261</v>
+        <v>3.874262102894468</v>
       </c>
       <c r="F30" t="n">
-        <v>97.03679583197658</v>
+        <v>40.20425614228279</v>
       </c>
       <c r="G30" t="inlineStr"/>
     </row>
@@ -889,19 +889,19 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>72.00020572956849</v>
+        <v>48.01693361878891</v>
       </c>
       <c r="C31" t="n">
-        <v>55.7683024939662</v>
+        <v>47.39379672986222</v>
       </c>
       <c r="D31" t="n">
-        <v>89.03791365329825</v>
+        <v>7.278793870489262</v>
       </c>
       <c r="E31" t="n">
-        <v>13.1797779352705</v>
+        <v>6.325113107755051</v>
       </c>
       <c r="F31" t="n">
-        <v>96.08689334495787</v>
+        <v>21.03577412659126</v>
       </c>
       <c r="G31" t="inlineStr"/>
     </row>
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>69.97548389308919</v>
+        <v>44.2579327985458</v>
       </c>
       <c r="C32" t="n">
-        <v>45.30973451327434</v>
+        <v>34.9550800599497</v>
       </c>
       <c r="D32" t="n">
-        <v>89.14797769498624</v>
+        <v>8.20975449003128</v>
       </c>
       <c r="E32" t="n">
-        <v>11.16229624379872</v>
+        <v>4.148346396482509</v>
       </c>
       <c r="F32" t="n">
-        <v>96.23946527172333</v>
+        <v>24.11458724085341</v>
       </c>
       <c r="G32" t="inlineStr"/>
     </row>
@@ -935,19 +935,19 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>67.39992113699876</v>
+        <v>39.47626731823149</v>
       </c>
       <c r="C33" t="n">
-        <v>39.97854652721909</v>
+        <v>28.61452397282506</v>
       </c>
       <c r="D33" t="n">
-        <v>88.1773686901892</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>9.492085991022915</v>
+        <v>2.346269037150322</v>
       </c>
       <c r="F33" t="n">
-        <v>96.71897704155768</v>
+        <v>33.79085702853434</v>
       </c>
       <c r="G33" t="inlineStr"/>
     </row>
@@ -958,19 +958,19 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>70.33859658146034</v>
+        <v>44.93207028688405</v>
       </c>
       <c r="C34" t="n">
-        <v>61.94690265486725</v>
+        <v>54.74220780870287</v>
       </c>
       <c r="D34" t="n">
-        <v>88.45301580344314</v>
+        <v>2.33152084363152</v>
       </c>
       <c r="E34" t="n">
-        <v>18.80226789510985</v>
+        <v>12.39151213917033</v>
       </c>
       <c r="F34" t="n">
-        <v>96.95727986050566</v>
+        <v>38.59966989271514</v>
       </c>
       <c r="G34" t="inlineStr"/>
     </row>
@@ -981,19 +981,19 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>71.66229491333642</v>
+        <v>47.38958470966958</v>
       </c>
       <c r="C35" t="n">
-        <v>68.70474658085278</v>
+        <v>62.7795324261848</v>
       </c>
       <c r="D35" t="n">
-        <v>88.89327197019504</v>
+        <v>6.055363321799327</v>
       </c>
       <c r="E35" t="n">
-        <v>27.73210489014883</v>
+        <v>22.02638118906519</v>
       </c>
       <c r="F35" t="n">
-        <v>96.78145887823308</v>
+        <v>35.05170430389913</v>
       </c>
       <c r="G35" t="inlineStr"/>
     </row>
@@ -1004,19 +1004,19 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>67.30653837581781</v>
+        <v>39.3028973917797</v>
       </c>
       <c r="C36" t="n">
-        <v>55.37563059686954</v>
+        <v>46.92677921071049</v>
       </c>
       <c r="D36" t="n">
-        <v>89.77616107428365</v>
+        <v>13.52315184495112</v>
       </c>
       <c r="E36" t="n">
-        <v>23.68851979057507</v>
+        <v>17.66354534467706</v>
       </c>
       <c r="F36" t="n">
-        <v>96.40782221427384</v>
+        <v>27.51193283116184</v>
       </c>
       <c r="G36" t="inlineStr"/>
     </row>
@@ -1027,19 +1027,19 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>63.58486630435404</v>
+        <v>32.39342068379177</v>
       </c>
       <c r="C37" t="n">
-        <v>49.9597747385358</v>
+        <v>40.48552485626466</v>
       </c>
       <c r="D37" t="n">
-        <v>89.88157563656138</v>
+        <v>14.41478552205194</v>
       </c>
       <c r="E37" t="n">
-        <v>20.78116387117096</v>
+        <v>14.52664670022728</v>
       </c>
       <c r="F37" t="n">
-        <v>96.26562045916886</v>
+        <v>24.64238377472693</v>
       </c>
       <c r="G37" t="inlineStr"/>
     </row>
@@ -1050,19 +1050,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>60.14846817192134</v>
+        <v>26.01356979970291</v>
       </c>
       <c r="C38" t="n">
-        <v>43.89916867792974</v>
+        <v>33.27744801677689</v>
       </c>
       <c r="D38" t="n">
-        <v>89.72735610912248</v>
+        <v>13.11034217608612</v>
       </c>
       <c r="E38" t="n">
-        <v>18.3557760453579</v>
+        <v>11.90976868667559</v>
       </c>
       <c r="F38" t="n">
-        <v>96.03191901579</v>
+        <v>19.92642400446839</v>
       </c>
       <c r="G38" t="inlineStr"/>
     </row>
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>57.82172389948968</v>
+        <v>21.6938487046931</v>
       </c>
       <c r="C39" t="n">
-        <v>40.10011620631089</v>
+        <v>28.75911076488558</v>
       </c>
       <c r="D39" t="n">
-        <v>89.55406206118455</v>
+        <v>11.64455978469815</v>
       </c>
       <c r="E39" t="n">
-        <v>17.15686274509804</v>
+        <v>10.61619830497674</v>
       </c>
       <c r="F39" t="n">
-        <v>95.95684394071492</v>
+        <v>18.41145247205361</v>
       </c>
       <c r="G39" t="inlineStr"/>
     </row>
@@ -1096,19 +1096,19 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>55.00108579494477</v>
+        <v>16.45718816319864</v>
       </c>
       <c r="C40" t="n">
-        <v>35.684276392241</v>
+        <v>23.50720817092251</v>
       </c>
       <c r="D40" t="n">
-        <v>89.28661293333658</v>
+        <v>9.382380403141708</v>
       </c>
       <c r="E40" t="n">
-        <v>15.64099535396488</v>
+        <v>8.980649546506935</v>
       </c>
       <c r="F40" t="n">
-        <v>95.77884335948853</v>
+        <v>14.81950383874793</v>
       </c>
       <c r="G40" t="inlineStr"/>
     </row>
@@ -1119,19 +1119,19 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>54.97984458568996</v>
+        <v>16.41775275949369</v>
       </c>
       <c r="C41" t="n">
-        <v>32.5175823320271</v>
+        <v>19.74095544224924</v>
       </c>
       <c r="D41" t="n">
-        <v>89.2275172672195</v>
+        <v>8.882528343405632</v>
       </c>
       <c r="E41" t="n">
-        <v>14.33628251144998</v>
+        <v>7.572926494862105</v>
       </c>
       <c r="F41" t="n">
-        <v>95.77345295347376</v>
+        <v>14.7107285674297</v>
       </c>
       <c r="G41" t="inlineStr"/>
     </row>
@@ -1142,19 +1142,19 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>52.40544399624789</v>
+        <v>11.63824490167635</v>
       </c>
       <c r="C42" t="n">
-        <v>26.76320729418075</v>
+        <v>12.89708916530481</v>
       </c>
       <c r="D42" t="n">
-        <v>88.82801275963668</v>
+        <v>5.503377821716883</v>
       </c>
       <c r="E42" t="n">
-        <v>10.7843137254902</v>
+        <v>3.740521251513414</v>
       </c>
       <c r="F42" t="n">
-        <v>95.68231826296343</v>
+        <v>12.8716832970716</v>
       </c>
       <c r="G42" t="inlineStr"/>
     </row>
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>52.29964021817131</v>
+        <v>11.44181471486794</v>
       </c>
       <c r="C43" t="n">
-        <v>25.52197065471402</v>
+        <v>11.42084586821629</v>
       </c>
       <c r="D43" t="n">
-        <v>88.61025014871167</v>
+        <v>3.661464585834353</v>
       </c>
       <c r="E43" t="n">
-        <v>9.827545476021735</v>
+        <v>2.708213853310394</v>
       </c>
       <c r="F43" t="n">
-        <v>95.50898825092375</v>
+        <v>9.373984044814767</v>
       </c>
       <c r="G43" t="inlineStr"/>
     </row>
@@ -1188,19 +1188,19 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>52.34580691300334</v>
+        <v>11.52752557184337</v>
       </c>
       <c r="C44" t="n">
-        <v>24.57955024326706</v>
+        <v>10.29999447598242</v>
       </c>
       <c r="D44" t="n">
-        <v>88.45858162097477</v>
+        <v>2.378598498222751</v>
       </c>
       <c r="E44" t="n">
-        <v>9.260571698558943</v>
+        <v>2.096476135856753</v>
       </c>
       <c r="F44" t="n">
-        <v>95.51210196371487</v>
+        <v>9.436816965513893</v>
       </c>
       <c r="G44" t="inlineStr"/>
     </row>
@@ -1211,19 +1211,19 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>49.32563799469818</v>
+        <v>5.920425753666474</v>
       </c>
       <c r="C45" t="n">
-        <v>24.2072021229332</v>
+        <v>9.85714868868555</v>
       </c>
       <c r="D45" t="n">
-        <v>88.82982476553084</v>
+        <v>5.518704408892601</v>
       </c>
       <c r="E45" t="n">
-        <v>8.028602557728721</v>
+        <v>0.7672400756683044</v>
       </c>
       <c r="F45" t="n">
-        <v>95.04445638292532</v>
+        <v>0</v>
       </c>
       <c r="G45" t="inlineStr"/>
     </row>
@@ -1234,19 +1234,19 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>48.91199060501637</v>
+        <v>5.152467978385538</v>
       </c>
       <c r="C46" t="n">
-        <v>26.85706623759721</v>
+        <v>13.00871867388095</v>
       </c>
       <c r="D46" t="n">
-        <v>88.6609077848394</v>
+        <v>4.089944801449922</v>
       </c>
       <c r="E46" t="n">
-        <v>8.227025750059063</v>
+        <v>0.9813292550818855</v>
       </c>
       <c r="F46" t="n">
-        <v>95.09862685265912</v>
+        <v>1.093128704329236</v>
       </c>
       <c r="G46" t="inlineStr"/>
     </row>
@@ -1257,19 +1257,19 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>48.14307634281404</v>
+        <v>3.724938877725907</v>
       </c>
       <c r="C47" t="n">
-        <v>26.85706623759721</v>
+        <v>13.00871867388095</v>
       </c>
       <c r="D47" t="n">
-        <v>88.614946307254</v>
+        <v>3.70118635689572</v>
       </c>
       <c r="E47" t="n">
-        <v>7.317505315379163</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>95.25392327811684</v>
+        <v>4.226920624203155</v>
       </c>
       <c r="G47" t="inlineStr"/>
     </row>
@@ -1280,19 +1280,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>47.76494110991102</v>
+        <v>3.022911258407645</v>
       </c>
       <c r="C48" t="n">
-        <v>40.56717618664521</v>
+        <v>29.31460046232398</v>
       </c>
       <c r="D48" t="n">
-        <v>88.84262303065721</v>
+        <v>5.626956665018885</v>
       </c>
       <c r="E48" t="n">
-        <v>24.40201984408221</v>
+        <v>18.43337793920857</v>
       </c>
       <c r="F48" t="n">
-        <v>95.31658674803838</v>
+        <v>5.491433153275203</v>
       </c>
       <c r="G48" t="inlineStr"/>
     </row>
@@ -1303,19 +1303,19 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>49.36146241799638</v>
+        <v>5.986935648574699</v>
       </c>
       <c r="C49" t="n">
-        <v>52.41767692179656</v>
+        <v>43.40878824341122</v>
       </c>
       <c r="D49" t="n">
-        <v>89.60787795889475</v>
+        <v>12.09975369458122</v>
       </c>
       <c r="E49" t="n">
-        <v>50.58316430020285</v>
+        <v>46.68158656286462</v>
       </c>
       <c r="F49" t="n">
-        <v>95.39033610919041</v>
+        <v>6.979652546560803</v>
       </c>
       <c r="G49" t="inlineStr"/>
     </row>
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>50.67878511791488</v>
+        <v>8.432613380844858</v>
       </c>
       <c r="C50" t="n">
-        <v>67.40987625943377</v>
+        <v>61.23950083848136</v>
       </c>
       <c r="D50" t="n">
-        <v>91.03068504777906</v>
+        <v>24.13435962620342</v>
       </c>
       <c r="E50" t="n">
-        <v>51.78360500826836</v>
+        <v>47.97680494487989</v>
       </c>
       <c r="F50" t="n">
-        <v>95.49238178270437</v>
+        <v>9.038875134419015</v>
       </c>
       <c r="G50" t="inlineStr"/>
     </row>
@@ -1349,19 +1349,19 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>50.62086244774101</v>
+        <v>8.325076947557392</v>
       </c>
       <c r="C51" t="n">
-        <v>78.12895069532237</v>
+        <v>73.98804634852357</v>
       </c>
       <c r="D51" t="n">
-        <v>90.7436975813044</v>
+        <v>21.70691806134212</v>
       </c>
       <c r="E51" t="n">
-        <v>53.05929600755965</v>
+        <v>49.35321480915058</v>
       </c>
       <c r="F51" t="n">
-        <v>95.79856354049903</v>
+        <v>15.21744566984281</v>
       </c>
       <c r="G51" t="inlineStr"/>
     </row>
@@ -1372,19 +1372,19 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>49.99877541923522</v>
+        <v>7.170140201045058</v>
       </c>
       <c r="C52" t="n">
-        <v>68.67409876259435</v>
+        <v>62.74308197440486</v>
       </c>
       <c r="D52" t="n">
-        <v>90.6320333670761</v>
+        <v>20.76242261610529</v>
       </c>
       <c r="E52" t="n">
-        <v>46.39735412237185</v>
+        <v>42.16529662907029</v>
       </c>
       <c r="F52" t="n">
-        <v>95.93349109478142</v>
+        <v>17.94020556680939</v>
       </c>
       <c r="G52" t="inlineStr"/>
     </row>
@@ -1395,19 +1395,19 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>48.41171874808659</v>
+        <v>4.223687398919098</v>
       </c>
       <c r="C53" t="n">
-        <v>62.06949392790101</v>
+        <v>54.88800961582272</v>
       </c>
       <c r="D53" t="n">
-        <v>90.54611105893156</v>
+        <v>20.03566132335282</v>
       </c>
       <c r="E53" t="n">
-        <v>41.58988896763525</v>
+        <v>36.97827056649462</v>
       </c>
       <c r="F53" t="n">
-        <v>95.93660480757256</v>
+        <v>18.00303848750883</v>
       </c>
       <c r="G53" t="inlineStr"/>
     </row>
@@ -1418,19 +1418,19 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>47.32980164240772</v>
+        <v>2.215052328951292</v>
       </c>
       <c r="C54" t="n">
-        <v>55.50319886603072</v>
+        <v>47.07850032196554</v>
       </c>
       <c r="D54" t="n">
-        <v>90.4494049793195</v>
+        <v>19.21768707482995</v>
       </c>
       <c r="E54" t="n">
-        <v>37.25490196078432</v>
+        <v>32.30102593513032</v>
       </c>
       <c r="F54" t="n">
-        <v>95.95424918005564</v>
+        <v>18.35909170480439</v>
       </c>
       <c r="G54" t="inlineStr"/>
     </row>
@@ -1441,19 +1441,19 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>47.23697842043777</v>
+        <v>2.042721215987444</v>
       </c>
       <c r="C55" t="n">
-        <v>64.06926406926407</v>
+        <v>57.26640159446534</v>
       </c>
       <c r="D55" t="n">
-        <v>90.63377268505472</v>
+        <v>20.77713438316501</v>
       </c>
       <c r="E55" t="n">
-        <v>36.61705646113867</v>
+        <v>31.61282100299497</v>
       </c>
       <c r="F55" t="n">
-        <v>96.24382446963094</v>
+        <v>24.20255332983243</v>
       </c>
       <c r="G55" t="inlineStr"/>
     </row>
@@ -1464,19 +1464,19 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>46.13670139214443</v>
+        <v>0</v>
       </c>
       <c r="C56" t="n">
-        <v>60.24594874152397</v>
+        <v>52.7192077349149</v>
       </c>
       <c r="D56" t="n">
-        <v>91.15243730628345</v>
+        <v>25.16418332038692</v>
       </c>
       <c r="E56" t="n">
-        <v>31.65603590833924</v>
+        <v>26.2601159752756</v>
       </c>
       <c r="F56" t="n">
-        <v>96.39951010918753</v>
+        <v>27.3441993647937</v>
       </c>
       <c r="G56" t="inlineStr"/>
     </row>
@@ -1487,19 +1487,19 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>46.60399262312548</v>
+        <v>0.867550341435821</v>
       </c>
       <c r="C57" t="n">
-        <v>55.20438263801096</v>
+        <v>46.7231084171109</v>
       </c>
       <c r="D57" t="n">
-        <v>91.37367855316572</v>
+        <v>27.03552009038899</v>
       </c>
       <c r="E57" t="n">
-        <v>62.01275690999292</v>
+        <v>59.013572930606</v>
       </c>
       <c r="F57" t="n">
-        <v>96.47112550338356</v>
+        <v>28.78935654087577</v>
       </c>
       <c r="G57" t="inlineStr"/>
     </row>
@@ -1510,19 +1510,19 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>47.22705931624309</v>
+        <v>2.024305885974153</v>
       </c>
       <c r="C58" t="n">
-        <v>61.29563651687545</v>
+        <v>53.96763570837864</v>
       </c>
       <c r="D58" t="n">
-        <v>91.11730308311505</v>
+        <v>24.86700562577972</v>
       </c>
       <c r="E58" t="n">
         <v>100</v>
       </c>
       <c r="F58" t="n">
-        <v>96.40262382197868</v>
+        <v>27.40703228549314</v>
       </c>
       <c r="G58" t="inlineStr"/>
     </row>
@@ -1533,19 +1533,19 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>48.17733398970863</v>
+        <v>3.788539971197721</v>
       </c>
       <c r="C59" t="n">
-        <v>55.04348159215415</v>
+        <v>46.5317435452661</v>
       </c>
       <c r="D59" t="n">
-        <v>91.59422407285655</v>
+        <v>28.90097215356731</v>
       </c>
       <c r="E59" t="n">
-        <v>85.81384360973307</v>
+        <v>84.69381252787869</v>
       </c>
       <c r="F59" t="n">
-        <v>96.70672977124592</v>
+        <v>33.54371420711762</v>
       </c>
       <c r="G59" t="inlineStr"/>
     </row>
@@ -1556,19 +1556,19 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>47.71823866099441</v>
+        <v>2.936205746261753</v>
       </c>
       <c r="C60" t="n">
-        <v>46.84519020802207</v>
+        <v>36.78124769412587</v>
       </c>
       <c r="D60" t="n">
-        <v>91.93478253307312</v>
+        <v>31.78153614386922</v>
       </c>
       <c r="E60" t="n">
-        <v>69.01724545239783</v>
+        <v>66.57108264831454</v>
       </c>
       <c r="F60" t="n">
-        <v>96.69427492008137</v>
+        <v>33.29238252432049</v>
       </c>
       <c r="G60" t="inlineStr"/>
     </row>
@@ -1579,19 +1579,19 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>48.18162002238534</v>
+        <v>3.796497212561491</v>
       </c>
       <c r="C61" t="n">
-        <v>42.90694556181282</v>
+        <v>32.09736464040056</v>
       </c>
       <c r="D61" t="n">
-        <v>91.75980714442252</v>
+        <v>30.3015323776569</v>
       </c>
       <c r="E61" t="n">
-        <v>61.56390266950154</v>
+        <v>58.52928057095521</v>
       </c>
       <c r="F61" t="n">
-        <v>96.69427492008137</v>
+        <v>33.29238252432049</v>
       </c>
       <c r="G61" t="inlineStr"/>
     </row>
@@ -1602,19 +1602,19 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>49.16814228648822</v>
+        <v>5.628026824747192</v>
       </c>
       <c r="C62" t="n">
-        <v>40.14097996398881</v>
+        <v>28.80771136725886</v>
       </c>
       <c r="D62" t="n">
-        <v>91.5963112544309</v>
+        <v>28.91862627403891</v>
       </c>
       <c r="E62" t="n">
-        <v>52.79943302622254</v>
+        <v>49.07283502198433</v>
       </c>
       <c r="F62" t="n">
-        <v>96.70257815419107</v>
+        <v>33.45993697951868</v>
       </c>
       <c r="G62" t="inlineStr"/>
     </row>
@@ -1625,19 +1625,19 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>48.97225037879096</v>
+        <v>5.26434336539683</v>
       </c>
       <c r="C63" t="n">
-        <v>36.08780599931043</v>
+        <v>23.98713911935869</v>
       </c>
       <c r="D63" t="n">
-        <v>91.64709933940702</v>
+        <v>29.34820987218418</v>
       </c>
       <c r="E63" t="n">
-        <v>45.1334750767777</v>
+        <v>40.80163130057988</v>
       </c>
       <c r="F63" t="n">
-        <v>96.54689251463446</v>
+        <v>30.31829094455741</v>
       </c>
       <c r="G63" t="inlineStr"/>
     </row>
@@ -1648,19 +1648,19 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>48.54287134799402</v>
+        <v>4.467178984650346</v>
       </c>
       <c r="C64" t="n">
-        <v>34.80825958702065</v>
+        <v>22.46533275754522</v>
       </c>
       <c r="D64" t="n">
-        <v>91.67284124549082</v>
+        <v>29.56594402466864</v>
       </c>
       <c r="E64" t="n">
-        <v>40.18426647767541</v>
+        <v>35.4616708086408</v>
       </c>
       <c r="F64" t="n">
-        <v>96.67455473907089</v>
+        <v>32.89444069322561</v>
       </c>
       <c r="G64" t="inlineStr"/>
     </row>
@@ -1671,19 +1671,19 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>50.01757171105503</v>
+        <v>7.205036489066058</v>
       </c>
       <c r="C65" t="n">
-        <v>32.64758839980079</v>
+        <v>19.8955759070578</v>
       </c>
       <c r="D65" t="n">
-        <v>91.94417485015775</v>
+        <v>31.86097968599196</v>
       </c>
       <c r="E65" t="n">
-        <v>36.54618473895582</v>
+        <v>31.53635378831326</v>
       </c>
       <c r="F65" t="n">
-        <v>96.63200066425874</v>
+        <v>32.0357241103361</v>
       </c>
       <c r="G65" t="inlineStr"/>
     </row>
@@ -1694,19 +1694,19 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>53.23301567708295</v>
+        <v>13.17467453414296</v>
       </c>
       <c r="C66" t="n">
-        <v>34.81592154158526</v>
+        <v>22.47444537049022</v>
       </c>
       <c r="D66" t="n">
-        <v>92.36195902862569</v>
+        <v>35.39474613374762</v>
       </c>
       <c r="E66" t="n">
-        <v>35.2586817859674</v>
+        <v>30.14719938826229</v>
       </c>
       <c r="F66" t="n">
-        <v>96.67040312201604</v>
+        <v>32.81066346562667</v>
       </c>
       <c r="G66" t="inlineStr"/>
     </row>
@@ -1717,19 +1717,19 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>52.66138259761285</v>
+        <v>12.11340815379777</v>
       </c>
       <c r="C67" t="n">
-        <v>35.39823008849557</v>
+        <v>23.16700395430952</v>
       </c>
       <c r="D67" t="n">
-        <v>91.78456444905704</v>
+        <v>30.51093842260378</v>
       </c>
       <c r="E67" t="n">
-        <v>33.32915054673734</v>
+        <v>28.06532702844304</v>
       </c>
       <c r="F67" t="n">
-        <v>96.77528063015957</v>
+        <v>34.92703083614409</v>
       </c>
       <c r="G67" t="inlineStr"/>
     </row>
@@ -1740,19 +1740,19 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>48.97778120660392</v>
+        <v>5.27461163331935</v>
       </c>
       <c r="C68" t="n">
-        <v>23.84911057477429</v>
+        <v>9.431258708559955</v>
       </c>
       <c r="D68" t="n">
-        <v>90.34951015007994</v>
+        <v>18.37274125336404</v>
       </c>
       <c r="E68" t="n">
-        <v>25.92133238837704</v>
+        <v>20.07264385394762</v>
       </c>
       <c r="F68" t="n">
-        <v>96.74271045238788</v>
+        <v>34.26978351297529</v>
       </c>
       <c r="G68" t="inlineStr"/>
     </row>
@@ -1763,19 +1763,19 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>50.47103499117077</v>
+        <v>8.046914524455453</v>
       </c>
       <c r="C69" t="n">
-        <v>23.16975060337892</v>
+        <v>8.623273694104098</v>
       </c>
       <c r="D69" t="n">
-        <v>90.40551618899195</v>
+        <v>18.8464601526884</v>
       </c>
       <c r="E69" t="n">
-        <v>26.00401606425703</v>
+        <v>20.16185560440961</v>
       </c>
       <c r="F69" t="n">
-        <v>96.71728179792697</v>
+        <v>33.75664799393176</v>
       </c>
       <c r="G69" t="inlineStr"/>
     </row>
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>50.93606953659415</v>
+        <v>8.91027521242408</v>
       </c>
       <c r="C70" t="n">
-        <v>24.30499687136855</v>
+        <v>9.973459178786911</v>
       </c>
       <c r="D70" t="n">
-        <v>90.38400662332285</v>
+        <v>18.66452463338269</v>
       </c>
       <c r="E70" t="n">
-        <v>26.293408929837</v>
+        <v>20.47409673102658</v>
       </c>
       <c r="F70" t="n">
-        <v>96.69790758500437</v>
+        <v>33.36568759846983</v>
       </c>
       <c r="G70" t="inlineStr"/>
     </row>
@@ -1809,19 +1809,19 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>50.52018149919708</v>
+        <v>8.138157558759977</v>
       </c>
       <c r="C71" t="n">
-        <v>26.76320729418075</v>
+        <v>12.89708916530481</v>
       </c>
       <c r="D71" t="n">
-        <v>90.33084147044261</v>
+        <v>18.21483495358923</v>
       </c>
       <c r="E71" t="n">
-        <v>24.03338845578392</v>
+        <v>18.03564221839887</v>
       </c>
       <c r="F71" t="n">
-        <v>96.87590816623074</v>
+        <v>36.95763623177552</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
@@ -1832,19 +1832,19 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>52.23216581803219</v>
+        <v>11.31654500082694</v>
       </c>
       <c r="C72" t="n">
-        <v>28.29176722982033</v>
+        <v>14.71505544783049</v>
       </c>
       <c r="D72" t="n">
-        <v>90.99155039325979</v>
+        <v>23.8033448673587</v>
       </c>
       <c r="E72" t="n">
-        <v>20.71226080793764</v>
+        <v>14.45230357484229</v>
       </c>
       <c r="F72" t="n">
-        <v>96.82989441053958</v>
+        <v>36.02910529255362</v>
       </c>
       <c r="G72" t="inlineStr"/>
     </row>
@@ -1855,19 +1855,19 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>52.93150348311588</v>
+        <v>12.61490155001477</v>
       </c>
       <c r="C73" t="n">
-        <v>36.69437740234201</v>
+        <v>24.70855431083714</v>
       </c>
       <c r="D73" t="n">
-        <v>91.22125632097141</v>
+        <v>25.74627890371827</v>
       </c>
       <c r="E73" t="n">
-        <v>19.55468934561777</v>
+        <v>13.20333906837444</v>
       </c>
       <c r="F73" t="n">
-        <v>96.88680616099971</v>
+        <v>37.17755145422292</v>
       </c>
       <c r="G73" t="inlineStr"/>
     </row>
@@ -1878,19 +1878,19 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>54.85993245212502</v>
+        <v>16.19512968095193</v>
       </c>
       <c r="C74" t="n">
-        <v>75.1407884151247</v>
+        <v>70.43412729997713</v>
       </c>
       <c r="D74" t="n">
-        <v>92.14819684905154</v>
+        <v>33.58666996210244</v>
       </c>
       <c r="E74" t="n">
-        <v>17.29466887156469</v>
+        <v>10.76488455574672</v>
       </c>
       <c r="F74" t="n">
-        <v>97.0878136200717</v>
+        <v>41.23376555713956</v>
       </c>
       <c r="G74" t="inlineStr"/>
     </row>
@@ -1901,19 +1901,19 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>56.66149485390343</v>
+        <v>19.53982346752161</v>
       </c>
       <c r="C75" t="n">
-        <v>69.6165191740413</v>
+        <v>63.86393336663871</v>
       </c>
       <c r="D75" t="n">
-        <v>92.80200647722013</v>
+        <v>39.11682319986811</v>
       </c>
       <c r="E75" t="n">
-        <v>15.08977084809827</v>
+        <v>8.385904543427007</v>
       </c>
       <c r="F75" t="n">
-        <v>97.44986922406278</v>
+        <v>48.53983794733315</v>
       </c>
       <c r="G75" t="inlineStr"/>
     </row>
@@ -1924,19 +1924,19 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>60.20832976163943</v>
+        <v>26.12470593741684</v>
       </c>
       <c r="C76" t="n">
-        <v>64.67328148744078</v>
+        <v>57.98477924829545</v>
       </c>
       <c r="D76" t="n">
-        <v>92.94810918742542</v>
+        <v>40.35261163288839</v>
       </c>
       <c r="E76" t="n">
-        <v>13.50500039373179</v>
+        <v>6.676012659572208</v>
       </c>
       <c r="F76" t="n">
-        <v>97.67267267267268</v>
+        <v>53.03588249514429</v>
       </c>
       <c r="G76" t="inlineStr"/>
     </row>
@@ -1947,19 +1947,19 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>63.82688428283244</v>
+        <v>32.84273957946576</v>
       </c>
       <c r="C77" t="n">
-        <v>75.96317153839277</v>
+        <v>71.41221442273947</v>
       </c>
       <c r="D77" t="n">
-        <v>92.78212027499777</v>
+        <v>38.94861866315155</v>
       </c>
       <c r="E77" t="n">
-        <v>14.44208205370502</v>
+        <v>7.687079164808089</v>
       </c>
       <c r="F77" t="n">
-        <v>98.00082340404923</v>
+        <v>59.65777419327984</v>
       </c>
       <c r="G77" t="inlineStr"/>
     </row>
@@ -1970,19 +1970,19 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>66.97140358998097</v>
+        <v>38.68070232668215</v>
       </c>
       <c r="C78" t="n">
         <v>100</v>
       </c>
       <c r="D78" t="n">
-        <v>92.55322602900949</v>
+        <v>37.01255011808639</v>
       </c>
       <c r="E78" t="n">
-        <v>19.83030159855107</v>
+        <v>13.5007115699144</v>
       </c>
       <c r="F78" t="n">
-        <v>98.24421195388938</v>
+        <v>64.56921416126934</v>
       </c>
       <c r="G78" t="inlineStr"/>
     </row>
@@ -1993,19 +1993,19 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>67.91675953070799</v>
+        <v>40.43580453015014</v>
       </c>
       <c r="C79" t="n">
-        <v>76.92857781353356</v>
+        <v>72.56040365380834</v>
       </c>
       <c r="D79" t="n">
-        <v>92.68593599077929</v>
+        <v>38.13505794474649</v>
       </c>
       <c r="E79" t="n">
-        <v>17.30844948421136</v>
+        <v>10.77975318082372</v>
       </c>
       <c r="F79" t="n">
-        <v>98.33987213019472</v>
+        <v>66.49958111386218</v>
       </c>
       <c r="G79" t="inlineStr"/>
     </row>
@@ -2016,19 +2016,19 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>70.04563196123141</v>
+        <v>44.38816631553276</v>
       </c>
       <c r="C80" t="n">
-        <v>64.37829623670332</v>
+        <v>57.6339436499133</v>
       </c>
       <c r="D80" t="n">
-        <v>92.85233074406862</v>
+        <v>39.54248366013066</v>
       </c>
       <c r="E80" t="n">
-        <v>16.15087802189149</v>
+        <v>9.53078867435587</v>
       </c>
       <c r="F80" t="n">
-        <v>98.25389906035069</v>
+        <v>64.7646943590003</v>
       </c>
       <c r="G80" t="inlineStr"/>
     </row>
@@ -2039,19 +2039,19 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>71.22686256693355</v>
+        <v>46.5811820353867</v>
       </c>
       <c r="C81" t="n">
-        <v>54.98346294806472</v>
+        <v>46.46036141053034</v>
       </c>
       <c r="D81" t="n">
-        <v>92.73910114365954</v>
+        <v>38.58474762453995</v>
       </c>
       <c r="E81" t="n">
-        <v>14.78659736987165</v>
+        <v>8.058794791733046</v>
       </c>
       <c r="F81" t="n">
-        <v>98.53966870095904</v>
+        <v>70.53136019206268</v>
       </c>
       <c r="G81" t="inlineStr"/>
     </row>
@@ -2062,19 +2062,19 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>73.35573499745695</v>
+        <v>50.53354382076931</v>
       </c>
       <c r="C82" t="n">
-        <v>55.5644945025476</v>
+        <v>47.15140122552547</v>
       </c>
       <c r="D82" t="n">
-        <v>92.64251101857937</v>
+        <v>37.76775416048764</v>
       </c>
       <c r="E82" t="n">
-        <v>14.46964327899835</v>
+        <v>7.716816414962087</v>
       </c>
       <c r="F82" t="n">
-        <v>98.64622687203334</v>
+        <v>72.68164236710291</v>
       </c>
       <c r="G82" t="inlineStr"/>
     </row>
@@ -2085,19 +2085,19 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>76.44553595409946</v>
+        <v>56.26991911990829</v>
       </c>
       <c r="C83" t="n">
-        <v>61.39268794136051</v>
+        <v>54.0830621390152</v>
       </c>
       <c r="D83" t="n">
-        <v>92.2987638087353</v>
+        <v>34.86021859724269</v>
       </c>
       <c r="E83" t="n">
-        <v>16.82612804157808</v>
+        <v>10.25935130312878</v>
       </c>
       <c r="F83" t="n">
-        <v>99.07730310956117</v>
+        <v>81.38051116612907</v>
       </c>
       <c r="G83" t="inlineStr"/>
     </row>
@@ -2108,19 +2108,19 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>78.17452153588553</v>
+        <v>59.47987028605154</v>
       </c>
       <c r="C84" t="n">
-        <v>50.40672208813803</v>
+        <v>41.01709394472246</v>
       </c>
       <c r="D84" t="n">
-        <v>91.76792396165614</v>
+        <v>30.37018729060244</v>
       </c>
       <c r="E84" t="n">
-        <v>15.25513819985826</v>
+        <v>8.564328044350985</v>
       </c>
       <c r="F84" t="n">
-        <v>99.23471858955732</v>
+        <v>84.557064379257</v>
       </c>
       <c r="G84" t="inlineStr"/>
     </row>
@@ -2131,19 +2131,19 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>74.41860023284353</v>
+        <v>52.50680810806191</v>
       </c>
       <c r="C85" t="n">
-        <v>49.26373973937427</v>
+        <v>39.65770768637135</v>
       </c>
       <c r="D85" t="n">
-        <v>91.75828443807606</v>
+        <v>30.28865278844731</v>
       </c>
       <c r="E85" t="n">
-        <v>15.44592151003518</v>
+        <v>8.77017415458584</v>
       </c>
       <c r="F85" t="n">
-        <v>99.37591008320433</v>
+        <v>87.40622694460168</v>
       </c>
       <c r="G85" t="inlineStr"/>
     </row>
@@ -2154,19 +2154,19 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>71.49555599640463</v>
+        <v>47.08002528564376</v>
       </c>
       <c r="C86" t="n">
-        <v>47.04440102670191</v>
+        <v>37.01817563069563</v>
       </c>
       <c r="D86" t="n">
-        <v>92.90636555593819</v>
+        <v>39.99952922345408</v>
       </c>
       <c r="E86" t="n">
-        <v>16.48948736120954</v>
+        <v>9.896132033390685</v>
       </c>
       <c r="F86" t="n">
-        <v>99.18939677004195</v>
+        <v>83.64249631130164</v>
       </c>
       <c r="G86" t="inlineStr"/>
     </row>
@@ -2177,19 +2177,19 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>72.46162776173577</v>
+        <v>48.87358748903664</v>
       </c>
       <c r="C87" t="n">
-        <v>43.30536719917252</v>
+        <v>32.57122051354009</v>
       </c>
       <c r="D87" t="n">
-        <v>93.58643888558417</v>
+        <v>45.75183014382219</v>
       </c>
       <c r="E87" t="n">
-        <v>15.7925820930782</v>
+        <v>9.144204422353914</v>
       </c>
       <c r="F87" t="n">
-        <v>99.21742018516213</v>
+        <v>84.2079925975944</v>
       </c>
       <c r="G87" t="inlineStr"/>
     </row>
@@ -2200,19 +2200,19 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>73.37247093457555</v>
+        <v>50.56461495371355</v>
       </c>
       <c r="C88" t="n">
-        <v>37.22177527487262</v>
+        <v>25.33580583521735</v>
       </c>
       <c r="D88" t="n">
-        <v>93.37389422859506</v>
+        <v>43.95405220911884</v>
       </c>
       <c r="E88" t="n">
-        <v>15.01299314906685</v>
+        <v>8.303065060855159</v>
       </c>
       <c r="F88" t="n">
-        <v>99.50595757047371</v>
+        <v>90.03050991572293</v>
       </c>
       <c r="G88" t="inlineStr"/>
     </row>
@@ -2223,19 +2223,19 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>72.93933671807457</v>
+        <v>49.76047887646667</v>
       </c>
       <c r="C89" t="n">
-        <v>35.40589204306019</v>
+        <v>23.17611656725451</v>
       </c>
       <c r="D89" t="n">
-        <v>93.38676518163696</v>
+        <v>44.06291928536111</v>
       </c>
       <c r="E89" t="n">
-        <v>59.21332388377037</v>
+        <v>55.99311795067865</v>
       </c>
       <c r="F89" t="n">
-        <v>99.3886743886744</v>
+        <v>87.66380323605192</v>
       </c>
       <c r="G89" t="inlineStr"/>
     </row>
@@ -2246,19 +2246,19 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>73.45304834889775</v>
+        <v>50.71421109135235</v>
       </c>
       <c r="C90" t="n">
-        <v>32.88510899130368</v>
+        <v>20.17806690835251</v>
       </c>
       <c r="D90" t="n">
-        <v>93.40728913378486</v>
+        <v>44.2365181366664</v>
       </c>
       <c r="E90" t="n">
-        <v>65.11930073234113</v>
+        <v>62.36538584082075</v>
       </c>
       <c r="F90" t="n">
-        <v>99.61597542242703</v>
+        <v>92.25060644709527</v>
       </c>
       <c r="G90" t="inlineStr"/>
     </row>
@@ -2269,19 +2269,19 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>72.90749761819042</v>
+        <v>49.70136794062157</v>
       </c>
       <c r="C91" t="n">
-        <v>30.9466344864575</v>
+        <v>17.87257583326983</v>
       </c>
       <c r="D91" t="n">
-        <v>92.90323478357665</v>
+        <v>39.97304804274641</v>
       </c>
       <c r="E91" t="n">
-        <v>46.45641389085755</v>
+        <v>42.22901930797172</v>
       </c>
       <c r="F91" t="n">
-        <v>99.85365549881681</v>
+        <v>97.04685272713674</v>
       </c>
       <c r="G91" t="inlineStr"/>
     </row>
@@ -2292,19 +2292,19 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>72.6847463770778</v>
+        <v>49.28781873945896</v>
       </c>
       <c r="C92" t="n">
-        <v>69.93832126575489</v>
+        <v>64.24666311032834</v>
       </c>
       <c r="D92" t="n">
-        <v>92.79504920530562</v>
+        <v>39.05797613162911</v>
       </c>
       <c r="E92" t="n">
-        <v>43.12544294826365</v>
+        <v>38.63506021793157</v>
       </c>
       <c r="F92" t="n">
-        <v>99.62220284800929</v>
+        <v>92.37627228849382</v>
       </c>
       <c r="G92" t="inlineStr"/>
     </row>
@@ -2315,19 +2315,19 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>73.72326594939128</v>
+        <v>51.21588404395187</v>
       </c>
       <c r="C93" t="n">
-        <v>56.56200268951383</v>
+        <v>48.33777030937114</v>
       </c>
       <c r="D93" t="n">
-        <v>92.94051966707777</v>
+        <v>40.28841678363052</v>
       </c>
       <c r="E93" t="n">
-        <v>40.30376551288882</v>
+        <v>35.59060457938148</v>
       </c>
       <c r="F93" t="n">
-        <v>99.44168326555895</v>
+        <v>88.73349166946439</v>
       </c>
       <c r="G93" t="inlineStr"/>
     </row>
@@ -2338,19 +2338,19 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>73.07029294376926</v>
+        <v>50.00360588331431</v>
       </c>
       <c r="C94" t="n">
-        <v>53.39208879031888</v>
+        <v>44.56768812097815</v>
       </c>
       <c r="D94" t="n">
-        <v>94.78775290741103</v>
+        <v>55.91296932127384</v>
       </c>
       <c r="E94" t="n">
-        <v>40.9991848687809</v>
+        <v>36.34092896184274</v>
       </c>
       <c r="F94" t="n">
-        <v>99.71567033467645</v>
+        <v>94.26239203416804</v>
       </c>
       <c r="G94" t="inlineStr"/>
     </row>
@@ -2361,19 +2361,19 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>73.71096855545011</v>
+        <v>51.19305329600473</v>
       </c>
       <c r="C95" t="n">
-        <v>54.69448097538096</v>
+        <v>46.11666570691566</v>
       </c>
       <c r="D95" t="n">
-        <v>95.12849895099869</v>
+        <v>58.7951199581199</v>
       </c>
       <c r="E95" t="n">
-        <v>32.05441692971147</v>
+        <v>26.68995013406453</v>
       </c>
       <c r="F95" t="n">
-        <v>99.42188349520812</v>
+        <v>88.33394377157853</v>
       </c>
       <c r="G95" t="inlineStr"/>
     </row>
@@ -2384,19 +2384,19 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>74.54891454274266</v>
+        <v>52.74874336503134</v>
       </c>
       <c r="C96" t="n">
-        <v>34.81313537628904</v>
+        <v>22.47113169305567</v>
       </c>
       <c r="D96" t="n">
-        <v>97.41951622293503</v>
+        <v>78.17335490345873</v>
       </c>
       <c r="E96" t="n">
-        <v>12.74080278332582</v>
+        <v>5.851479814393217</v>
       </c>
       <c r="F96" t="n">
-        <v>99.30715172650658</v>
+        <v>86.01872313047217</v>
       </c>
       <c r="G96" t="inlineStr"/>
     </row>
@@ -2407,19 +2407,19 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>74.91085052032437</v>
+        <v>53.42069622892244</v>
       </c>
       <c r="C97" t="n">
-        <v>20.16626441405202</v>
+        <v>5.051129419667679</v>
       </c>
       <c r="D97" t="n">
-        <v>97.54790951372146</v>
+        <v>79.25935079914311</v>
       </c>
       <c r="E97" t="n">
-        <v>10.25277580911883</v>
+        <v>3.167017141400625</v>
       </c>
       <c r="F97" t="n">
-        <v>99.12089508863703</v>
+        <v>82.26017205591837</v>
       </c>
       <c r="G97" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Remove unnamed column from data file and visualizations
Update app.py and preprocess_typical_day.py to remove the 'Unnamed: 6' column from the typical day averages data file and all associated visualizations and selections.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 8877ae72-82e6-4518-9133-e997a155a908
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9d9f6885-c530-4d92-b5a9-0a657be3b603
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/296373d1-a774-4ae0-bc03-ad5165af73dc/8877ae72-82e6-4518-9133-e997a155a908/ToRk9hW
</commit_message>
<xml_diff>
--- a/attached_assets/typical_day_averages.xlsx
+++ b/attached_assets/typical_day_averages.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,11 +457,6 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Temperature</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 6</t>
         </is>
       </c>
     </row>
@@ -476,7 +471,6 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -489,7 +483,6 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -502,7 +495,6 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -515,7 +507,6 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -538,7 +529,6 @@
       <c r="F6" t="n">
         <v>41.42767643925939</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -561,7 +551,6 @@
       <c r="F7" t="n">
         <v>21.67589523561039</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -584,7 +573,6 @@
       <c r="F8" t="n">
         <v>24.84839699918508</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -607,7 +595,6 @@
       <c r="F9" t="n">
         <v>34.81911682756259</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -630,7 +617,6 @@
       <c r="F10" t="n">
         <v>39.77426243924106</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -653,7 +639,6 @@
       <c r="F11" t="n">
         <v>36.11833183550299</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -676,7 +661,6 @@
       <c r="F12" t="n">
         <v>28.34912421994373</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -699,7 +683,6 @@
       <c r="F13" t="n">
         <v>25.39225444436933</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -722,7 +705,6 @@
       <c r="F14" t="n">
         <v>20.53278745730665</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -745,7 +727,6 @@
       <c r="F15" t="n">
         <v>18.97171516094443</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -768,7 +749,6 @@
       <c r="F16" t="n">
         <v>15.27046310344078</v>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -791,7 +771,6 @@
       <c r="F17" t="n">
         <v>15.15837778767679</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -814,7 +793,6 @@
       <c r="F18" t="n">
         <v>13.26337015097488</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -837,7 +815,6 @@
       <c r="F19" t="n">
         <v>9.659235494396993</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -860,7 +837,6 @@
       <c r="F20" t="n">
         <v>9.723980428347392</v>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -883,7 +859,6 @@
       <c r="F21" t="n">
         <v>0</v>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -906,7 +881,6 @@
       <c r="F22" t="n">
         <v>1.126392740836994</v>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -929,7 +903,6 @@
       <c r="F23" t="n">
         <v>4.355546321618323</v>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -952,7 +925,6 @@
       <c r="F24" t="n">
         <v>5.658538117372312</v>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -975,7 +947,6 @@
       <c r="F25" t="n">
         <v>7.192044203829311</v>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -998,7 +969,6 @@
       <c r="F26" t="n">
         <v>9.313929179994437</v>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1021,7 +991,6 @@
       <c r="F27" t="n">
         <v>15.68051435179374</v>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1044,7 +1013,6 @@
       <c r="F28" t="n">
         <v>18.48612815631563</v>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1067,7 +1035,6 @@
       <c r="F29" t="n">
         <v>18.55087309026635</v>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1090,7 +1057,6 @@
       <c r="F30" t="n">
         <v>18.91776104931915</v>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1113,7 +1079,6 @@
       <c r="F31" t="n">
         <v>24.93903990671589</v>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1136,7 +1101,6 @@
       <c r="F32" t="n">
         <v>28.17628660424098</v>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1159,7 +1123,6 @@
       <c r="F33" t="n">
         <v>29.66542008510241</v>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1182,7 +1145,6 @@
       <c r="F34" t="n">
         <v>28.2410315381917</v>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1205,7 +1167,6 @@
       <c r="F35" t="n">
         <v>34.56445342069085</v>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1228,7 +1189,6 @@
       <c r="F36" t="n">
         <v>34.3054736848886</v>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1251,7 +1211,6 @@
       <c r="F37" t="n">
         <v>34.3054736848886</v>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1274,7 +1233,6 @@
       <c r="F38" t="n">
         <v>34.47812684209021</v>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1297,7 +1255,6 @@
       <c r="F39" t="n">
         <v>31.24088014456511</v>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1320,7 +1277,6 @@
       <c r="F40" t="n">
         <v>33.89542243653565</v>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1343,7 +1299,6 @@
       <c r="F41" t="n">
         <v>33.0105750058787</v>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1366,7 +1321,6 @@
       <c r="F42" t="n">
         <v>33.80909585793501</v>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1389,7 +1343,6 @@
       <c r="F43" t="n">
         <v>35.98986453929342</v>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1412,7 +1365,6 @@
       <c r="F44" t="n">
         <v>35.3126171018966</v>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1435,7 +1387,6 @@
       <c r="F45" t="n">
         <v>34.78386680796765</v>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1458,7 +1409,6 @@
       <c r="F46" t="n">
         <v>34.38100944116444</v>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1481,7 +1431,6 @@
       <c r="F47" t="n">
         <v>38.08226149866809</v>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1504,7 +1453,6 @@
       <c r="F48" t="n">
         <v>37.12547525251066</v>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1527,7 +1475,6 @@
       <c r="F49" t="n">
         <v>38.30886876749497</v>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1550,7 +1497,6 @@
       <c r="F50" t="n">
         <v>42.48851394807733</v>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1573,7 +1519,6 @@
       <c r="F51" t="n">
         <v>50.01691099021102</v>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1596,7 +1541,6 @@
       <c r="F52" t="n">
         <v>54.64977070844682</v>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1619,7 +1563,6 @@
       <c r="F53" t="n">
         <v>61.47316735867524</v>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1642,7 +1585,6 @@
       <c r="F54" t="n">
         <v>66.53406302913952</v>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1665,7 +1607,6 @@
       <c r="F55" t="n">
         <v>68.52317127772989</v>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1688,7 +1629,6 @@
       <c r="F56" t="n">
         <v>66.7354917125411</v>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1711,7 +1651,6 @@
       <c r="F57" t="n">
         <v>72.67763787288729</v>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1734,7 +1673,6 @@
       <c r="F58" t="n">
         <v>74.89335339030455</v>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1757,7 +1695,6 @@
       <c r="F59" t="n">
         <v>83.85692980167406</v>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1780,7 +1717,6 @@
       <c r="F60" t="n">
         <v>87.13014590694988</v>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1803,7 +1739,6 @@
       <c r="F61" t="n">
         <v>90.06600882808506</v>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1826,7 +1761,6 @@
       <c r="F62" t="n">
         <v>86.18774742389262</v>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1849,7 +1783,6 @@
       <c r="F63" t="n">
         <v>86.77045182944684</v>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1872,7 +1805,6 @@
       <c r="F64" t="n">
         <v>92.77014904219367</v>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1895,7 +1827,6 @@
       <c r="F65" t="n">
         <v>90.33142319672457</v>
       </c>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1918,7 +1849,6 @@
       <c r="F66" t="n">
         <v>95.05780337511108</v>
       </c>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1941,7 +1871,6 @@
       <c r="F67" t="n">
         <v>100</v>
       </c>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1964,7 +1893,6 @@
       <c r="F68" t="n">
         <v>95.18729324301221</v>
       </c>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1987,7 +1915,6 @@
       <c r="F69" t="n">
         <v>91.4336623764124</v>
       </c>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2010,7 +1937,6 @@
       <c r="F70" t="n">
         <v>97.13080783691393</v>
       </c>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2033,7 +1959,6 @@
       <c r="F71" t="n">
         <v>91.021956188465</v>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2056,7 +1981,6 @@
       <c r="F72" t="n">
         <v>88.63628310783868</v>
       </c>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2079,7 +2003,6 @@
       <c r="F73" t="n">
         <v>84.76335887698126</v>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>